<commit_message>
Add ConeTec method-specific CPT interpreted-property codes
Add four codes reflecting the methods ConeTec's SCREENzW/IFI3 output
actually uses, so real interpreted values can be encoded without
mislabeling the method:
- sbt_robertson_2009_qtn: SBTn from the Qtn-Fr chart polygons (vs the
  existing Ic-band variant)
- n60_ic_rw1998: equivalent SPT N60 via Ic (Robertson & Wride 1998)
- gamma_sbt_qtn_zone: unit weight assigned per SBT Qtn zone [PROVISIONAL
  citation - confirm with ConeTec]
- ocr_pkr2015: OCR per Robertson 2015 [PROVISIONAL citation - confirm]

Supports the C-030-S (Project Squash) worked example for ConeTec.
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/cpt_interpreted_properties.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/cpt_interpreted_properties.xlsx
@@ -1007,7 +1007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="7" customWidth="1" style="2" min="1" max="1"/>
@@ -1507,6 +1507,154 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>sbt_robertson_2009_qtn</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Soil Behaviour Type Zone (Robertson 2009, Qtn-Fr chart)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Numeric normalized soil behaviour type (SBTn) zone assigned from the normalized cone resistance (Qtn) versus normalized friction ratio (Fr) chart polygons per Robertson (2009). This chart-polygon variant is distinct from the Ic-band variant (sbt_robertson_2009_ic); ConeTec's SCREENzW 'SBT Qtn' output uses this chart.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Robertson, P.K. 2009. "Interpretation of cone penetration tests - a unified approach." Canadian Geotechnical Journal 46(11): 1337-1355.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1139/T09-065</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>n60_ic_rw1998</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Equivalent SPT N60 (Ic, Robertson &amp; Wride 1998)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Equivalent SPT blow count at 60% energy ratio estimated from corrected tip resistance using a soil behaviour type index (Ic) dependent qt/N60 ratio per Robertson and Wride (1998). Distinct from n60_ic_based (Jefferies &amp; Davies 1993) and from SBT-zone-based N60.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Robertson, P.K. and Wride, C.E. 1998. "Evaluating cyclic liquefaction potential using the cone penetration test." Canadian Geotechnical Journal 35(3): 442-459.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1139/t98-017</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>gamma_sbt_qtn_zone</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Soil Unit Weight (SBT Qtn zone assigned)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Total soil unit weight assigned per normalized soil behaviour type (Qtn) zone, as used in ConeTec SCREENzW ('SBT Qtn zone assigned unit weights'). PROVISIONAL AUTHORITY - pending ConeTec/Jim Greig confirmation of the exact zone-unit-weight table and reference; one of the nine unit-weight methods to be registered.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>force per volume</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Robertson, P.K. 2010. "Soil behaviour type from the CPT: an update." 2nd International Symposium on Cone Penetration Testing (CPT'10), Huntington Beach, California. [PROVISIONAL - confirm with ConeTec]</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.cpt-robertson.com/publications/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ocr_pkr2015</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Overconsolidation Ratio (Robertson 2015)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Overconsolidation ratio estimated from CPT per Robertson (2015), corresponding to ConeTec SCREENzW 'OCR (PKR2015)'. PROVISIONAL AUTHORITY - pending ConeTec/Jim Greig confirmation of reference; ConeTec also reports an 'OCR (JS1978)' variant whose citation is to be resolved.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Robertson, P.K. and Cabal, K.L. 2015. Guide to Cone Penetration Testing for Geotechnical Engineering, 6th ed. Gregg Drilling &amp; Testing, Inc. [PROVISIONAL - confirm with ConeTec]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.cpt-robertson.com/publications/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -1522,7 +1670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="6.83203125" customWidth="1" min="1" max="1"/>
@@ -1752,6 +1900,74 @@
         </is>
       </c>
       <c r="D13" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>sbt_robertson_2009_qtn</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>//diggs:propertyClass</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>n60_ic_rw1998</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>//diggs:propertyClass</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>gamma_sbt_qtn_zone</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>//diggs:propertyClass</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ocr_pkr2015</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>//diggs:propertyClass</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
         </is>

</xml_diff>